<commit_message>
Testimonios como conversacion con polaroid (opcion 2)
- Cada testimonio: inicial automatica del nombre (sin fotos ni logos de la
  persona), nombre, @instagram como texto, "Pedido real", el texto en uno o
  dos globos, estrellas y la respuesta de Heart Graphic.
- La foto del pedido va como polaroid con el producto abajo en Neulis (hasta
  dos lineas); lado_foto derecha por defecto o izquierda; en celular arriba.
- Columna opcional "respuesta" en la pestana testimonios y en el Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pestanas_planners_y_testimonios.xlsx
+++ b/pestanas_planners_y_testimonios.xlsx
@@ -265,12 +265,26 @@
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">• lado_foto: izquierda o derecha (dónde va la foto al lado del texto).</t>
+          <t xml:space="preserve">• lado_foto: derecha (por defecto) o izquierda: dónde va la polaroid con la foto, al lado de la conversación.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• respuesta: opcional, lo que contesta Heart Graphic. Vacío = ¡Gracias, (nombre)! Nos encantó hacerlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• El círculo de la persona muestra solo la inicial de su nombre (no se usan fotos ni logos personales). El producto va escrito bajo la foto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">• Se muestran en el orden de la pestaña. Si la pestaña queda vacía, la web muestra los testimonios de siempre.</t>
         </is>
@@ -864,6 +878,7 @@
     <col min="5" max="5" width="70" customWidth="1"/>
     <col min="6" max="6" width="50" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -902,6 +917,11 @@
           <t xml:space="preserve">lado_foto</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">respuesta</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
@@ -926,7 +946,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">izquierda</t>
+          <t xml:space="preserve">derecha</t>
         </is>
       </c>
     </row>
@@ -980,7 +1000,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">izquierda</t>
+          <t xml:space="preserve">derecha</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1032,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G5"/>
+  <autoFilter ref="A1:H5"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elige una opción de la lista" sqref="A2:A300">
       <formula1>"si,no"</formula1>

</xml_diff>

<commit_message>
Testimonios: origen sin Instagram (WhatsApp o texto libre)
En la columna instagram: @usuario (o el enlace) sale con el icono de
Instagram; un texto que nombra WhatsApp ("Pedido directo de WhatsApp") con el
icono de WhatsApp; cualquier otro texto ("Pedido personalizado") sin icono.
Nunca es un enlace. Texto del origen mas oscuro para que se lea mejor y sin
puntito de navegacion cuando hay un solo testimonio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pestanas_planners_y_testimonios.xlsx
+++ b/pestanas_planners_y_testimonios.xlsx
@@ -237,54 +237,61 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">• instagram: el usuario (ej. @vetpelitos). Se muestra como texto, SIN enlace a su perfil.</t>
+          <t xml:space="preserve">• instagram: el usuario (ej. @vetpelitos) y se ve con el ícono de Instagram, SIN enlace a su perfil.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">• producto: qué pidió (opcional).</t>
+          <t xml:space="preserve">  Si la persona no tiene Instagram escribe otra cosa: 'Pedido directo de WhatsApp' sale con el ícono de WhatsApp; 'Pedido personalizado' (o cualquier texto) sale sin ícono. Vacío = no se muestra nada.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">• texto: el testimonio, sin comillas.</t>
+          <t xml:space="preserve">• producto: qué pidió (opcional).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">• foto: opcional, la foto del pedido subida a Cloudinary (https://...).</t>
+          <t xml:space="preserve">• texto: el testimonio, sin comillas.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">• lado_foto: derecha (por defecto) o izquierda: dónde va la polaroid con la foto, al lado de la conversación.</t>
+          <t xml:space="preserve">• foto: opcional, la foto del pedido subida a Cloudinary (https://...).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">• respuesta: opcional, lo que contesta Heart Graphic. Vacío = ¡Gracias, (nombre)! Nos encantó hacerlo.</t>
+          <t xml:space="preserve">• lado_foto: derecha (por defecto) o izquierda: dónde va la polaroid con la foto, al lado de la conversación.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">• El círculo de la persona muestra solo la inicial de su nombre (no se usan fotos ni logos personales). El producto va escrito bajo la foto.</t>
+          <t xml:space="preserve">• respuesta: opcional, lo que contesta Heart Graphic. Vacío = ¡Gracias, (nombre)! Nos encantó hacerlo.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• El círculo de la persona muestra solo la inicial de su nombre (no se usan fotos ni logos personales). El producto va escrito bajo la foto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">• Se muestran en el orden de la pestaña. Si la pestaña queda vacía, la web muestra los testimonios de siempre.</t>
         </is>

</xml_diff>